<commit_message>
Korp Filial 08/2026: TXT corrigido; skill com regras de rescisão e consignado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VLoTgLZUjFbc7Wvyz5oBv
</commit_message>
<xml_diff>
--- a/Korp/Filial/2026-08/Fechamento_Folha_Korp_Filial_08-2026.xlsx
+++ b/Korp/Filial/2026-08/Fechamento_Folha_Korp_Filial_08-2026.xlsx
@@ -708,7 +708,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Folha 08/2026. Outros meses no TXT de 08: rescisão de estágio da Isabele (07); parte das férias do Matheus e da Ana de 09 (férias pagas integralmente em 08); férias da Fernanda lançadas no TXT de 07. Faltam no TXT de 08: rescisões de Guilherme, Enzo e Wellington (devem vir no TXT de 09). Consignado da Ana depende de confirmação.</t>
+          <t>Folha 08/2026. Outros meses no TXT de 08: rescisão de estágio da Isabele (07); parte das férias do Matheus e da Ana de 09 (férias pagas integralmente em 08); férias da Fernanda lançadas no TXT de 07. Faltam no TXT de 08: rescisões de Guilherme, Enzo e Wellington (devem vir no TXT de 09). Consignado da Ana: estorno e provisão excluídos (confirmado).</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Correções: -3.800,00 e -3.900,00 bolsas (CC 7 e 13) para 2526; +3.339,00 salário do Bruno com D/C na mesma conta; -3.329,46 verbas e descontos da rescisão Alyson/Wendel para 2523; +1.730,46 afastamento invertido (CC 8); +94,98 diferença de férias da Fernanda; +2,62 horas extras Isabele; -70,00 contribuição do CC 14 invertida; -1.378,95 consignado da Ana (exclusão do estorno 459,65 e da provisão 919,30 - a confirmar)</t>
+          <t>Correções: -3.800,00 e -3.900,00 bolsas (CC 7 e 13) para 2526; +3.339,00 salário do Bruno com D/C na mesma conta; -3.329,46 verbas e descontos da rescisão Alyson/Wendel para 2523; +1.730,46 afastamento invertido (CC 8); +94,98 diferença de férias da Fernanda; +2,62 horas extras Isabele; -70,00 contribuição do CC 14 invertida; -1.378,95 consignado da Ana (exclusão do estorno 459,65 e da provisão 919,30)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Folha = Ana 919,30 + Jhonatan 475,32 + Enzo (rescisão) 2.416,71. Correção: +1.378,95 exclusão do estorno 459,65 e da provisão 919,30 do consignado da Ana (a confirmar). Outros meses: -2.416,71 consignado da rescisão do Enzo (TXT de 09)</t>
+          <t>Folha = Ana 919,30 + Jhonatan 475,32 + Enzo (rescisão) 2.416,71. Correção: +1.378,95 exclusão do estorno 459,65 e da provisão 919,30 do consignado da Ana (confirmado). Outros meses: -2.416,71 consignado da rescisão do Enzo (TXT de 09)</t>
         </is>
       </c>
     </row>

</xml_diff>